<commit_message>
feat: update multi-step instructor registration, Step 6 submit fix, mobile responsiveness, success modal, and documentation
</commit_message>
<xml_diff>
--- a/public/templates/Template_Import_Siswa.xlsx
+++ b/public/templates/Template_Import_Siswa.xlsx
@@ -7,7 +7,7 @@
     <workbookView activeTab="0" autoFilterDateGrouping="true" firstSheet="0" minimized="false" showHorizontalScroll="true" showSheetTabs="true" showVerticalScroll="true" tabRatio="600" visibility="visible"/>
   </bookViews>
   <sheets>
-    <sheet name="Worksheet" sheetId="1" r:id="rId4"/>
+    <sheet name="Import Siswa" sheetId="1" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="999999" calcMode="auto" calcCompleted="1" fullCalcOnLoad="0" forceFullCalc="0"/>
@@ -15,15 +15,15 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="11">
+  <si>
+    <t>NISN</t>
+  </si>
   <si>
     <t>Nama Lengkap</t>
   </si>
   <si>
-    <t>NISN</t>
-  </si>
-  <si>
-    <t>Sekolah Kodlan</t>
+    <t>Kode Sekolah</t>
   </si>
   <si>
     <t>Kelas</t>
@@ -32,19 +32,22 @@
     <t>No HP Orangtua</t>
   </si>
   <si>
-    <t>Andi Siswa Contoh</t>
-  </si>
-  <si>
-    <t>0123456789</t>
-  </si>
-  <si>
-    <t>KODLAN001</t>
-  </si>
-  <si>
-    <t>X IPA 1</t>
+    <t>Ahmad Fauzi</t>
+  </si>
+  <si>
+    <t>X-IPA-1</t>
   </si>
   <si>
     <t>081234567890</t>
+  </si>
+  <si>
+    <t>Budi Santoso</t>
+  </si>
+  <si>
+    <t>X-IPA-2</t>
+  </si>
+  <si>
+    <t>081234567891</t>
   </si>
 </sst>
 </file>
@@ -384,8 +387,15 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col min="1" max="1" width="12.854" bestFit="true" customWidth="true" style="0"/>
+    <col min="2" max="2" width="15.282" bestFit="true" customWidth="true" style="0"/>
+    <col min="3" max="3" width="15.282" bestFit="true" customWidth="true" style="0"/>
+    <col min="4" max="4" width="9.283" bestFit="true" customWidth="true" style="0"/>
+    <col min="5" max="5" width="17.567" bestFit="true" customWidth="true" style="0"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" t="s">
@@ -405,20 +415,37 @@
       </c>
     </row>
     <row r="2" spans="1:5">
-      <c r="A2" t="s">
+      <c r="A2">
+        <v>1234567890</v>
+      </c>
+      <c r="B2" t="s">
         <v>5</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2">
+        <v>20218093</v>
+      </c>
+      <c r="D2" t="s">
         <v>6</v>
       </c>
-      <c r="C2" t="s">
+      <c r="E2" t="s">
         <v>7</v>
       </c>
-      <c r="D2" t="s">
+    </row>
+    <row r="3" spans="1:5">
+      <c r="A3">
+        <v>1234567891</v>
+      </c>
+      <c r="B3" t="s">
         <v>8</v>
       </c>
-      <c r="E2" t="s">
+      <c r="C3">
+        <v>20218094</v>
+      </c>
+      <c r="D3" t="s">
         <v>9</v>
+      </c>
+      <c r="E3" t="s">
+        <v>10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>